<commit_message>
Avances de las correcciones en la metodologia, pendiente justificar rangos
</commit_message>
<xml_diff>
--- a/CORRECCIONES TESIS AGOSTO 2026/CONTROL DE CORRECCIONES.xlsx
+++ b/CORRECCIONES TESIS AGOSTO 2026/CONTROL DE CORRECCIONES.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Angeal\Desktop\GNLPDA\CORRECCIONES TESIS AGOSTO 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{775CD2A7-4D02-46B2-86B5-0EEF71D1676C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EB0FE55-68CE-4668-A70F-29DA9EF898DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-34510" yWindow="-110" windowWidth="34620" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="77040" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="83">
   <si>
     <t>Director(es) que lo solicita</t>
   </si>
@@ -601,7 +601,27 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="5">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -1114,7 +1134,9 @@
       <c r="C14" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="D14" s="2"/>
+      <c r="D14" s="2" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="15" spans="1:4" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
@@ -1126,7 +1148,9 @@
       <c r="C15" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D15" s="2"/>
+      <c r="D15" s="2" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="16" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
@@ -1138,7 +1162,9 @@
       <c r="C16" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D16" s="2"/>
+      <c r="D16" s="2" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="17" spans="1:4" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
@@ -1188,7 +1214,7 @@
       </c>
       <c r="D20" s="2"/>
     </row>
-    <row r="21" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>4</v>
       </c>
@@ -1237,17 +1263,27 @@
       <c r="D24" s="2"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A15:D24 A2:D12">
-    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
+  <conditionalFormatting sqref="A13 C13:D13">
+    <cfRule type="cellIs" dxfId="4" priority="3" operator="equal">
       <formula>$D$2</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A14:D14">
+  <conditionalFormatting sqref="A2:D12">
+    <cfRule type="cellIs" dxfId="3" priority="5" operator="equal">
+      <formula>$D$2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A17:D24 A14:C16">
+    <cfRule type="cellIs" dxfId="2" priority="4" operator="equal">
+      <formula>$D$2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D14">
     <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
       <formula>$D$2</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A13 C13:D13">
+  <conditionalFormatting sqref="D15:D16">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>$D$2</formula>
     </cfRule>

</xml_diff>

<commit_message>
Justificación del algoritmo genetico lista
</commit_message>
<xml_diff>
--- a/CORRECCIONES TESIS AGOSTO 2026/CONTROL DE CORRECCIONES.xlsx
+++ b/CORRECCIONES TESIS AGOSTO 2026/CONTROL DE CORRECCIONES.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Angeal\Desktop\GNLPDA\CORRECCIONES TESIS AGOSTO 2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Angel\Desktop\GNLPDA\CORRECCIONES TESIS AGOSTO 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EB0FE55-68CE-4668-A70F-29DA9EF898DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13BEF656-F39A-41B9-BE5A-7CB2EF563BC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="77040" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -601,27 +601,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="5">
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="3">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -934,15 +914,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D24"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="29.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="29.44140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="58" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="33.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.42578125" customWidth="1"/>
+    <col min="3" max="3" width="33.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -956,7 +936,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -970,7 +950,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -984,7 +964,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>1</v>
       </c>
@@ -998,7 +978,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>9</v>
       </c>
@@ -1012,7 +992,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" ht="42.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>1</v>
       </c>
@@ -1026,7 +1006,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>1</v>
       </c>
@@ -1040,7 +1020,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="58.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
         <v>1</v>
       </c>
@@ -1054,7 +1034,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>1</v>
       </c>
@@ -1068,7 +1048,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>1</v>
       </c>
@@ -1082,7 +1062,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>1</v>
       </c>
@@ -1096,7 +1076,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>20</v>
       </c>
@@ -1110,7 +1090,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>1</v>
       </c>
@@ -1124,7 +1104,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>1</v>
       </c>
@@ -1138,7 +1118,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>22</v>
       </c>
@@ -1152,7 +1132,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="1" t="s">
         <v>20</v>
       </c>
@@ -1166,7 +1146,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" ht="42.6" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>20</v>
       </c>
@@ -1178,7 +1158,7 @@
       </c>
       <c r="D17" s="2"/>
     </row>
-    <row r="18" spans="1:4" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" ht="42" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>22</v>
       </c>
@@ -1190,7 +1170,7 @@
       </c>
       <c r="D18" s="2"/>
     </row>
-    <row r="19" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>1</v>
       </c>
@@ -1202,7 +1182,7 @@
       </c>
       <c r="D19" s="2"/>
     </row>
-    <row r="20" spans="1:4" ht="58.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="1" t="s">
         <v>33</v>
       </c>
@@ -1214,7 +1194,7 @@
       </c>
       <c r="D20" s="2"/>
     </row>
-    <row r="21" spans="1:4" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A21" s="1" t="s">
         <v>4</v>
       </c>
@@ -1226,7 +1206,7 @@
       </c>
       <c r="D21" s="2"/>
     </row>
-    <row r="22" spans="1:4" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" ht="42" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A22" s="1" t="s">
         <v>4</v>
       </c>
@@ -1238,7 +1218,7 @@
       </c>
       <c r="D22" s="2"/>
     </row>
-    <row r="23" spans="1:4" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>38</v>
       </c>
@@ -1250,7 +1230,7 @@
       </c>
       <c r="D23" s="2"/>
     </row>
-    <row r="24" spans="1:4" ht="72" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" ht="69.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A24" s="1" t="s">
         <v>9</v>
       </c>
@@ -1264,26 +1244,16 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A13 C13:D13">
-    <cfRule type="cellIs" dxfId="4" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
       <formula>$D$2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A2:D12">
-    <cfRule type="cellIs" dxfId="3" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="5" operator="equal">
       <formula>$D$2</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A17:D24 A14:C16">
-    <cfRule type="cellIs" dxfId="2" priority="4" operator="equal">
-      <formula>$D$2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D14">
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
-      <formula>$D$2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D15:D16">
+  <conditionalFormatting sqref="A14:D24">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>$D$2</formula>
     </cfRule>
@@ -1295,12 +1265,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80CD9C86-BB81-45D2-B52F-9BBB3BE4D29C}">
   <dimension ref="B2:D9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="4" max="4" width="46.5703125" customWidth="1"/>
+    <col min="4" max="4" width="46.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B2" s="5" t="s">
         <v>46</v>
       </c>
@@ -1311,7 +1281,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B3" s="5" t="s">
         <v>45</v>
       </c>
@@ -1322,7 +1292,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B4" s="5" t="s">
         <v>45</v>
       </c>
@@ -1333,7 +1303,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="5" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B5" s="5" t="s">
         <v>45</v>
       </c>
@@ -1344,7 +1314,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="6" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B6" s="5" t="s">
         <v>45</v>
       </c>
@@ -1355,7 +1325,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B7" s="5" t="s">
         <v>45</v>
       </c>
@@ -1366,7 +1336,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="8" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B8" s="5" t="s">
         <v>45</v>
       </c>
@@ -1377,7 +1347,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="9" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B9" s="5" t="s">
         <v>45</v>
       </c>
@@ -1397,9 +1367,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0E9ECB9-9509-4435-9143-07DA83ABD06A}">
   <dimension ref="B2:D16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B2" s="5" t="s">
         <v>46</v>
       </c>
@@ -1410,7 +1380,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="3" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B3" s="5" t="s">
         <v>59</v>
       </c>
@@ -1421,7 +1391,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="4" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B4" s="5" t="s">
         <v>59</v>
       </c>
@@ -1432,7 +1402,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="5" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B5" s="5" t="s">
         <v>59</v>
       </c>
@@ -1443,7 +1413,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="6" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B6" s="5" t="s">
         <v>59</v>
       </c>
@@ -1454,7 +1424,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="7" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B7" s="5" t="s">
         <v>59</v>
       </c>
@@ -1465,7 +1435,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="8" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B8" s="5" t="s">
         <v>59</v>
       </c>
@@ -1476,7 +1446,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="9" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B9" s="5" t="s">
         <v>59</v>
       </c>
@@ -1487,7 +1457,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="10" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B10" s="5" t="s">
         <v>59</v>
       </c>
@@ -1498,7 +1468,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="11" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B11" s="5" t="s">
         <v>59</v>
       </c>
@@ -1509,7 +1479,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="12" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B12" s="5" t="s">
         <v>59</v>
       </c>
@@ -1520,7 +1490,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="13" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B13" s="5" t="s">
         <v>59</v>
       </c>
@@ -1531,7 +1501,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="14" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B14" s="5" t="s">
         <v>59</v>
       </c>
@@ -1542,7 +1512,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="15" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B15" s="5" t="s">
         <v>59</v>
       </c>
@@ -1553,7 +1523,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="16" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B16" s="5" t="s">
         <v>59</v>
       </c>
@@ -1572,12 +1542,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9318431B-ADA9-43B9-8F56-BA9994346673}">
   <dimension ref="B1:D22"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="4" max="4" width="206.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="206.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B1" s="11" t="s">
         <v>46</v>
       </c>
@@ -1588,7 +1558,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="2" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B2" s="12" t="s">
         <v>59</v>
       </c>
@@ -1599,7 +1569,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="3" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B3" s="12" t="s">
         <v>59</v>
       </c>
@@ -1610,7 +1580,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="4" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B4" s="12" t="s">
         <v>59</v>
       </c>
@@ -1621,7 +1591,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="5" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B5" s="12" t="s">
         <v>59</v>
       </c>
@@ -1632,7 +1602,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="6" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B6" s="12" t="s">
         <v>59</v>
       </c>
@@ -1643,7 +1613,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="7" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B7" s="12" t="s">
         <v>59</v>
       </c>
@@ -1654,7 +1624,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="8" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B8" s="8" t="s">
         <v>45</v>
       </c>
@@ -1665,7 +1635,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="9" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B9" s="12" t="s">
         <v>59</v>
       </c>
@@ -1676,7 +1646,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="10" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B10" s="12" t="s">
         <v>59</v>
       </c>
@@ -1687,7 +1657,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="11" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B11" s="8" t="s">
         <v>45</v>
       </c>
@@ -1698,7 +1668,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="12" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B12" s="8" t="s">
         <v>45</v>
       </c>
@@ -1709,7 +1679,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="13" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B13" s="8" t="s">
         <v>45</v>
       </c>
@@ -1720,7 +1690,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="14" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B14" s="12" t="s">
         <v>59</v>
       </c>
@@ -1731,7 +1701,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="15" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B15" s="8" t="s">
         <v>45</v>
       </c>
@@ -1742,7 +1712,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="16" spans="2:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B16" s="8" t="s">
         <v>45</v>
       </c>
@@ -1753,7 +1723,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="17" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B17" s="8" t="s">
         <v>45</v>
       </c>
@@ -1764,7 +1734,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="18" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B18" s="12" t="s">
         <v>59</v>
       </c>
@@ -1775,7 +1745,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="19" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B19" s="12" t="s">
         <v>59</v>
       </c>
@@ -1786,7 +1756,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="20" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B20" s="12" t="s">
         <v>59</v>
       </c>
@@ -1797,7 +1767,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="21" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B21" s="12" t="s">
         <v>59</v>
       </c>
@@ -1808,7 +1778,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="22" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="B22" s="12" t="s">
         <v>59</v>
       </c>

</xml_diff>

<commit_message>
Correcciones hasta reordenar resultados, pendientes unas pocas más
</commit_message>
<xml_diff>
--- a/CORRECCIONES TESIS AGOSTO 2026/CONTROL DE CORRECCIONES.xlsx
+++ b/CORRECCIONES TESIS AGOSTO 2026/CONTROL DE CORRECCIONES.xlsx
@@ -1,25 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Angel\Desktop\GNLPDA\CORRECCIONES TESIS AGOSTO 2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Angeal\Desktop\GNLPDA\CORRECCIONES TESIS AGOSTO 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13BEF656-F39A-41B9-BE5A-7CB2EF563BC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C601618-1710-4299-BFFC-C9BC062DBC55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="77040" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
-    <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
-    <sheet name="Hoja3" sheetId="3" r:id="rId3"/>
-    <sheet name="Hoja4" sheetId="4" r:id="rId4"/>
+    <sheet name="Hoja5" sheetId="5" r:id="rId2"/>
+    <sheet name="Hoja2" sheetId="2" r:id="rId3"/>
+    <sheet name="Hoja3" sheetId="3" r:id="rId4"/>
+    <sheet name="Hoja4" sheetId="4" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Hoja4!$B$1:$D$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Hoja4!$B$1:$D$22</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -31,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="122">
   <si>
     <t>Director(es) que lo solicita</t>
   </si>
@@ -414,6 +415,124 @@
   </si>
   <si>
     <t>Incluir el diagrama del esquema general de un algoritmo genético (Población -&gt; Selección -&gt; Cruza -&gt; Muta, etc.).</t>
+  </si>
+  <si>
+    <t>Dataset</t>
+  </si>
+  <si>
+    <t>#Samples</t>
+  </si>
+  <si>
+    <t>#Features</t>
+  </si>
+  <si>
+    <t>#Classes</t>
+  </si>
+  <si>
+    <t>Reference</t>
+  </si>
+  <si>
+    <t>Iris</t>
+  </si>
+  <si>
+    <t>[47]</t>
+  </si>
+  <si>
+    <t>Diabetes</t>
+  </si>
+  <si>
+    <t>[48]</t>
+  </si>
+  <si>
+    <t>Golub</t>
+  </si>
+  <si>
+    <t>[49]</t>
+  </si>
+  <si>
+    <t>[50]</t>
+  </si>
+  <si>
+    <t>SRBCT</t>
+  </si>
+  <si>
+    <t>[51]</t>
+  </si>
+  <si>
+    <t>Wine</t>
+  </si>
+  <si>
+    <t>[52]</t>
+  </si>
+  <si>
+    <t>Synthetical</t>
+  </si>
+  <si>
+    <t>(Generated)</t>
+  </si>
+  <si>
+    <t>Colon Cancer</t>
+  </si>
+  <si>
+    <t>Muestras</t>
+  </si>
+  <si>
+    <t>Variables</t>
+  </si>
+  <si>
+    <t>Clases</t>
+  </si>
+  <si>
+    <t>Referencia</t>
+  </si>
+  <si>
+    <t>penguins</t>
+  </si>
+  <si>
+    <t>[35]</t>
+  </si>
+  <si>
+    <t>wines</t>
+  </si>
+  <si>
+    <t>[9]</t>
+  </si>
+  <si>
+    <t>[71]</t>
+  </si>
+  <si>
+    <t>Ionosphere</t>
+  </si>
+  <si>
+    <t>[76]</t>
+  </si>
+  <si>
+    <t>Cebolla3D</t>
+  </si>
+  <si>
+    <t>Sintéticos</t>
+  </si>
+  <si>
+    <t>Cebolla10D</t>
+  </si>
+  <si>
+    <t>Cebolla20D</t>
+  </si>
+  <si>
+    <t>pimadiabetes</t>
+  </si>
+  <si>
+    <t>[78]</t>
+  </si>
+  <si>
+    <t>Indicadores</t>
+  </si>
+  <si>
+    <t>[58]</t>
+  </si>
+  <si>
+    <t>Breast Cancer
+WDBC</t>
   </si>
 </sst>
 </file>
@@ -496,7 +615,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -512,6 +631,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -558,7 +689,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
@@ -597,6 +728,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -914,15 +1050,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D24"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="29.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="29.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="58" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="33.5546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.44140625" customWidth="1"/>
+    <col min="3" max="3" width="33.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -936,7 +1072,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -950,7 +1086,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
@@ -964,7 +1100,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>1</v>
       </c>
@@ -978,7 +1114,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>9</v>
       </c>
@@ -992,7 +1128,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="42.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:4" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>1</v>
       </c>
@@ -1006,7 +1142,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>1</v>
       </c>
@@ -1020,7 +1156,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" ht="58.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>1</v>
       </c>
@@ -1034,7 +1170,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>1</v>
       </c>
@@ -1048,7 +1184,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>1</v>
       </c>
@@ -1062,7 +1198,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>1</v>
       </c>
@@ -1076,7 +1212,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>20</v>
       </c>
@@ -1090,7 +1226,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>1</v>
       </c>
@@ -1104,7 +1240,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>1</v>
       </c>
@@ -1118,7 +1254,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>22</v>
       </c>
@@ -1132,7 +1268,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>20</v>
       </c>
@@ -1146,7 +1282,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="42.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>20</v>
       </c>
@@ -1156,9 +1292,11 @@
       <c r="C17" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D17" s="2"/>
-    </row>
-    <row r="18" spans="1:4" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D17" s="2" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>22</v>
       </c>
@@ -1170,7 +1308,7 @@
       </c>
       <c r="D18" s="2"/>
     </row>
-    <row r="19" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>1</v>
       </c>
@@ -1182,7 +1320,7 @@
       </c>
       <c r="D19" s="2"/>
     </row>
-    <row r="20" spans="1:4" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" ht="58.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>33</v>
       </c>
@@ -1194,7 +1332,7 @@
       </c>
       <c r="D20" s="2"/>
     </row>
-    <row r="21" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:4" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>4</v>
       </c>
@@ -1206,7 +1344,7 @@
       </c>
       <c r="D21" s="2"/>
     </row>
-    <row r="22" spans="1:4" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" ht="43.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>4</v>
       </c>
@@ -1218,7 +1356,7 @@
       </c>
       <c r="D22" s="2"/>
     </row>
-    <row r="23" spans="1:4" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" ht="57.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>38</v>
       </c>
@@ -1230,7 +1368,7 @@
       </c>
       <c r="D23" s="2"/>
     </row>
-    <row r="24" spans="1:4" ht="69.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:4" ht="72" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>9</v>
       </c>
@@ -1263,14 +1401,334 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D8E058B-C30B-45F0-BBCF-B7D4D02421F4}">
+  <dimension ref="B2:L12"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="8" max="8" width="13.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C2" t="s">
+        <v>84</v>
+      </c>
+      <c r="D2" t="s">
+        <v>85</v>
+      </c>
+      <c r="E2" t="s">
+        <v>86</v>
+      </c>
+      <c r="F2" t="s">
+        <v>87</v>
+      </c>
+      <c r="H2" t="s">
+        <v>83</v>
+      </c>
+      <c r="I2" t="s">
+        <v>102</v>
+      </c>
+      <c r="J2" t="s">
+        <v>103</v>
+      </c>
+      <c r="K2" t="s">
+        <v>104</v>
+      </c>
+      <c r="L2" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="3" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B3" t="s">
+        <v>88</v>
+      </c>
+      <c r="C3">
+        <v>150</v>
+      </c>
+      <c r="D3">
+        <v>4</v>
+      </c>
+      <c r="E3">
+        <v>3</v>
+      </c>
+      <c r="F3" t="s">
+        <v>89</v>
+      </c>
+      <c r="H3" t="s">
+        <v>106</v>
+      </c>
+      <c r="I3">
+        <v>342</v>
+      </c>
+      <c r="J3">
+        <v>4</v>
+      </c>
+      <c r="K3">
+        <v>3</v>
+      </c>
+      <c r="L3" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="4" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B4" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="C4" s="18">
+        <v>768</v>
+      </c>
+      <c r="D4" s="18">
+        <v>8</v>
+      </c>
+      <c r="E4" s="18">
+        <v>2</v>
+      </c>
+      <c r="F4" s="18" t="s">
+        <v>91</v>
+      </c>
+      <c r="H4" s="17" t="s">
+        <v>108</v>
+      </c>
+      <c r="I4" s="17">
+        <v>178</v>
+      </c>
+      <c r="J4" s="17">
+        <v>13</v>
+      </c>
+      <c r="K4" s="17">
+        <v>3</v>
+      </c>
+      <c r="L4" s="17" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="5" spans="2:12" ht="30" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>92</v>
+      </c>
+      <c r="C5">
+        <v>72</v>
+      </c>
+      <c r="D5">
+        <v>7129</v>
+      </c>
+      <c r="E5">
+        <v>2</v>
+      </c>
+      <c r="F5" t="s">
+        <v>93</v>
+      </c>
+      <c r="H5" s="16" t="s">
+        <v>121</v>
+      </c>
+      <c r="I5">
+        <v>569</v>
+      </c>
+      <c r="J5">
+        <v>30</v>
+      </c>
+      <c r="K5">
+        <v>2</v>
+      </c>
+      <c r="L5" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="6" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>101</v>
+      </c>
+      <c r="C6">
+        <v>62</v>
+      </c>
+      <c r="D6">
+        <v>2000</v>
+      </c>
+      <c r="E6">
+        <v>2</v>
+      </c>
+      <c r="F6" t="s">
+        <v>94</v>
+      </c>
+      <c r="H6" t="s">
+        <v>111</v>
+      </c>
+      <c r="I6">
+        <v>351</v>
+      </c>
+      <c r="J6">
+        <v>34</v>
+      </c>
+      <c r="K6">
+        <v>2</v>
+      </c>
+      <c r="L6" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="7" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>95</v>
+      </c>
+      <c r="C7">
+        <v>83</v>
+      </c>
+      <c r="D7">
+        <v>2308</v>
+      </c>
+      <c r="E7">
+        <v>4</v>
+      </c>
+      <c r="F7" t="s">
+        <v>96</v>
+      </c>
+      <c r="H7" t="s">
+        <v>113</v>
+      </c>
+      <c r="I7">
+        <v>300</v>
+      </c>
+      <c r="J7">
+        <v>3</v>
+      </c>
+      <c r="K7">
+        <v>3</v>
+      </c>
+      <c r="L7" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="8" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B8" s="17" t="s">
+        <v>97</v>
+      </c>
+      <c r="C8" s="17">
+        <v>178</v>
+      </c>
+      <c r="D8" s="17">
+        <v>13</v>
+      </c>
+      <c r="E8" s="17">
+        <v>3</v>
+      </c>
+      <c r="F8" s="17" t="s">
+        <v>98</v>
+      </c>
+      <c r="H8" t="s">
+        <v>115</v>
+      </c>
+      <c r="I8">
+        <v>300</v>
+      </c>
+      <c r="J8">
+        <v>10</v>
+      </c>
+      <c r="K8">
+        <v>3</v>
+      </c>
+      <c r="L8" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="9" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>99</v>
+      </c>
+      <c r="C9">
+        <v>45</v>
+      </c>
+      <c r="D9">
+        <v>110</v>
+      </c>
+      <c r="E9">
+        <v>3</v>
+      </c>
+      <c r="F9" t="s">
+        <v>100</v>
+      </c>
+      <c r="H9" t="s">
+        <v>116</v>
+      </c>
+      <c r="I9">
+        <v>300</v>
+      </c>
+      <c r="J9">
+        <v>20</v>
+      </c>
+      <c r="K9">
+        <v>3</v>
+      </c>
+      <c r="L9" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="10" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="H10" s="18" t="s">
+        <v>117</v>
+      </c>
+      <c r="I10" s="18">
+        <v>768</v>
+      </c>
+      <c r="J10" s="18">
+        <v>8</v>
+      </c>
+      <c r="K10" s="18">
+        <v>2</v>
+      </c>
+      <c r="L10" s="18" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="11" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="H11" t="s">
+        <v>119</v>
+      </c>
+      <c r="I11">
+        <v>2446</v>
+      </c>
+      <c r="J11">
+        <v>12</v>
+      </c>
+      <c r="K11">
+        <v>5</v>
+      </c>
+      <c r="L11" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="12" spans="2:12" x14ac:dyDescent="0.25">
+      <c r="H12" t="s">
+        <v>119</v>
+      </c>
+      <c r="I12">
+        <v>2470</v>
+      </c>
+      <c r="J12">
+        <v>12</v>
+      </c>
+      <c r="K12">
+        <v>5</v>
+      </c>
+      <c r="L12" t="s">
+        <v>120</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{80CD9C86-BB81-45D2-B52F-9BBB3BE4D29C}">
   <dimension ref="B2:D9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="46.5546875" customWidth="1"/>
+    <col min="4" max="4" width="46.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B2" s="5" t="s">
         <v>46</v>
       </c>
@@ -1281,7 +1739,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="3" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B3" s="5" t="s">
         <v>45</v>
       </c>
@@ -1292,7 +1750,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="4" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B4" s="5" t="s">
         <v>45</v>
       </c>
@@ -1303,7 +1761,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="5" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B5" s="5" t="s">
         <v>45</v>
       </c>
@@ -1314,7 +1772,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="6" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B6" s="5" t="s">
         <v>45</v>
       </c>
@@ -1325,7 +1783,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="7" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B7" s="5" t="s">
         <v>45</v>
       </c>
@@ -1336,7 +1794,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="8" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B8" s="5" t="s">
         <v>45</v>
       </c>
@@ -1347,7 +1805,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="9" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B9" s="5" t="s">
         <v>45</v>
       </c>
@@ -1364,12 +1822,12 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0E9ECB9-9509-4435-9143-07DA83ABD06A}">
   <dimension ref="B2:D16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B2" s="5" t="s">
         <v>46</v>
       </c>
@@ -1380,7 +1838,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="3" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B3" s="5" t="s">
         <v>59</v>
       </c>
@@ -1391,7 +1849,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="4" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B4" s="5" t="s">
         <v>59</v>
       </c>
@@ -1402,7 +1860,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="5" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B5" s="5" t="s">
         <v>59</v>
       </c>
@@ -1413,7 +1871,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="6" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B6" s="5" t="s">
         <v>59</v>
       </c>
@@ -1424,7 +1882,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="7" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B7" s="5" t="s">
         <v>59</v>
       </c>
@@ -1435,7 +1893,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="8" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B8" s="5" t="s">
         <v>59</v>
       </c>
@@ -1446,7 +1904,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="9" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B9" s="5" t="s">
         <v>59</v>
       </c>
@@ -1457,7 +1915,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="10" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B10" s="5" t="s">
         <v>59</v>
       </c>
@@ -1468,7 +1926,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="11" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B11" s="5" t="s">
         <v>59</v>
       </c>
@@ -1479,7 +1937,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="12" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B12" s="5" t="s">
         <v>59</v>
       </c>
@@ -1490,7 +1948,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="13" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B13" s="5" t="s">
         <v>59</v>
       </c>
@@ -1501,7 +1959,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="14" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B14" s="5" t="s">
         <v>59</v>
       </c>
@@ -1512,7 +1970,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="15" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B15" s="5" t="s">
         <v>59</v>
       </c>
@@ -1523,7 +1981,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="16" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B16" s="5" t="s">
         <v>59</v>
       </c>
@@ -1539,15 +1997,15 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9318431B-ADA9-43B9-8F56-BA9994346673}">
   <dimension ref="B1:D22"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="206.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="206.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B1" s="11" t="s">
         <v>46</v>
       </c>
@@ -1558,7 +2016,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="2" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B2" s="12" t="s">
         <v>59</v>
       </c>
@@ -1569,7 +2027,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="3" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B3" s="12" t="s">
         <v>59</v>
       </c>
@@ -1580,7 +2038,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="4" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B4" s="12" t="s">
         <v>59</v>
       </c>
@@ -1591,7 +2049,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="5" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B5" s="12" t="s">
         <v>59</v>
       </c>
@@ -1602,7 +2060,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="6" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B6" s="12" t="s">
         <v>59</v>
       </c>
@@ -1613,7 +2071,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="7" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B7" s="12" t="s">
         <v>59</v>
       </c>
@@ -1624,7 +2082,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="8" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B8" s="8" t="s">
         <v>45</v>
       </c>
@@ -1635,7 +2093,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="9" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B9" s="12" t="s">
         <v>59</v>
       </c>
@@ -1646,7 +2104,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="10" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B10" s="12" t="s">
         <v>59</v>
       </c>
@@ -1657,7 +2115,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="11" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B11" s="8" t="s">
         <v>45</v>
       </c>
@@ -1668,7 +2126,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="12" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B12" s="8" t="s">
         <v>45</v>
       </c>
@@ -1679,7 +2137,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="13" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B13" s="8" t="s">
         <v>45</v>
       </c>
@@ -1690,7 +2148,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="14" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B14" s="12" t="s">
         <v>59</v>
       </c>
@@ -1701,7 +2159,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="15" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B15" s="8" t="s">
         <v>45</v>
       </c>
@@ -1712,7 +2170,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="16" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B16" s="8" t="s">
         <v>45</v>
       </c>
@@ -1723,7 +2181,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="17" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B17" s="8" t="s">
         <v>45</v>
       </c>
@@ -1734,7 +2192,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="18" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B18" s="12" t="s">
         <v>59</v>
       </c>
@@ -1745,7 +2203,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="19" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B19" s="12" t="s">
         <v>59</v>
       </c>
@@ -1756,7 +2214,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="20" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B20" s="12" t="s">
         <v>59</v>
       </c>
@@ -1767,7 +2225,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="21" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B21" s="12" t="s">
         <v>59</v>
       </c>
@@ -1778,7 +2236,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="22" spans="2:4" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:4" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B22" s="12" t="s">
         <v>59</v>
       </c>

</xml_diff>